<commit_message>
fix: open first galaxy after clearing60 without extra planet conquests
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/galaxy.xlsx
+++ b/space-battleship/config_excel/galaxy.xlsx
@@ -803,11 +803,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>conquered_planet_count</t>
+          <t>stage_cleared</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="H4" t="n">
         <v>200</v>

</xml_diff>